<commit_message>
Added new warehouse tabs for computer equipment with exact functionalities to warehouse 1. Pending event functions for unstaging, unwarehousing, unpulling an item. File name changes as well to the qr code folders, qr label folders, and excel.
</commit_message>
<xml_diff>
--- a/activity_log.xlsx
+++ b/activity_log.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -453,12 +453,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-04-11 13:06:49</t>
+          <t>2026-04-13 15:29:05</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Enzo Maverick</t>
+          <t>Mark Benjamin</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -468,217 +468,217 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Session started by 'Enzo Maverick'</t>
+          <t>Session started by 'Mark Benjamin'</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-04-11 13:07:35</t>
+          <t>2026-04-13 15:43:09</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Enzo Maverick</t>
+          <t>Mark Benjamin</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>PUT WAREHOUSE</t>
+          <t>LOGIN</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Hostname: PS-2044 | Shelf: Area C</t>
+          <t>Session started by 'Mark Benjamin'</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-04-11 13:07:51</t>
+          <t>2026-04-13 15:44:24</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Enzo Maverick</t>
+          <t>Mark Benjamin</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>UNSTAGE</t>
+          <t>LOGIN</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Hostname: PS-2044 | Shelf: Area C</t>
+          <t>Session started by 'Mark Benjamin'</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-11 13:07:56</t>
+          <t>2026-04-13 15:45:36</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Enzo Maverick</t>
+          <t>Mark Benjamin</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>PUT WAREHOUSE</t>
+          <t>LOGIN</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Hostname: PS-2044 | Shelf: Area C</t>
+          <t>Session started by 'Mark Benjamin'</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-04-11 13:09:38</t>
+          <t>2026-04-13 15:46:13</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Enzo Maverick</t>
+          <t>Mark Benjamin</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>UNSTAGE</t>
+          <t>LOGIN</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Hostname: PS-2000 | Shelf: Area B</t>
+          <t>Session started by 'Mark Benjamin'</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-04-11 13:09:41</t>
+          <t>2026-04-13 16:09:09</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Enzo Maverick</t>
+          <t>Mark Benjamin</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>UNSTAGE</t>
+          <t>LOGIN</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Hostname: PS-2012 | Shelf: Area B</t>
+          <t>Session started by 'Mark Benjamin'</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-04-11 13:09:44</t>
+          <t>2026-04-13 16:10:38</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Enzo Maverick</t>
+          <t>Mark Benjamin</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>UNSTAGE</t>
+          <t>LOGIN</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Hostname: PS-2121 | Shelf: Area B</t>
+          <t>Session started by 'Mark Benjamin'</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-04-11 13:09:46</t>
+          <t>2026-04-13 16:17:42</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Enzo Maverick</t>
+          <t>Mark Benjamin</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>UNSTAGE</t>
+          <t>PUT WAREHOUSE</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Hostname: PS-2122 | Shelf: Area B</t>
+          <t>[W2] Set: SET-001 | Items: 1</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-04-11 13:09:48</t>
+          <t>2026-04-13 16:19:34</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Enzo Maverick</t>
+          <t>Mark Benjamin</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>UNSTAGE</t>
+          <t>PUT WAREHOUSE</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Hostname: PS-2044 | Shelf: Area C</t>
+          <t>[W2] Set: SET-002 | Items: 2</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-04-11 13:09:54</t>
+          <t>2026-04-13 16:27:20</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Enzo Maverick</t>
+          <t>Mark Benjamin</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>PUT WAREHOUSE</t>
+          <t>LOGIN</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Hostname: PS-2000 | Shelf: Area B</t>
+          <t>Session started by 'Mark Benjamin'</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-04-11 13:09:54</t>
+          <t>2026-04-13 16:28:12</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Enzo Maverick</t>
+          <t>Mark Benjamin</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -688,19 +688,19 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Hostname: PS-2012 | Shelf: Area B</t>
+          <t>[W1] Hostname: PS-0142 | Shelf: Area A</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-04-11 13:09:54</t>
+          <t>2026-04-13 16:28:12</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Enzo Maverick</t>
+          <t>Mark Benjamin</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -710,117 +710,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Hostname: PS-2121 | Shelf: Area B</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>2026-04-11 13:09:54</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Enzo Maverick</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>PUT WAREHOUSE</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Hostname: PS-2122 | Shelf: Area B</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>2026-04-11 13:09:54</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Enzo Maverick</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>PUT WAREHOUSE</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Hostname: PS-2044 | Shelf: Area C</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>2026-04-11 13:10:50</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Enzo Maverick</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>PUT WAREHOUSE</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Hostname: PS-1987 | Shelf: Area C</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>2026-04-11 13:10:50</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Enzo Maverick</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>PUT WAREHOUSE</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Hostname: PS-1900 | Shelf: Area C</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>2026-04-11 13:12:01</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Enzo Maverick</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>SHELF STATUS</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Shelf: Area B → FULL</t>
+          <t>[W1] Hostname: PS-0111 | Shelf: Area A</t>
         </is>
       </c>
     </row>

</xml_diff>